<commit_message>
update status tracker (minor errors)
</commit_message>
<xml_diff>
--- a/docs/StatusTracker.xlsx
+++ b/docs/StatusTracker.xlsx
@@ -255,7 +255,7 @@
     <t>setup FunctionGemma</t>
   </si>
   <si>
-    <t>Week 5</t>
+    <t>Week 5 (February 12 - February 18)</t>
   </si>
   <si>
     <t>Implement Conversation Summarizer</t>
@@ -273,7 +273,7 @@
     <t>Train Model Based on the Architecture Diagram</t>
   </si>
   <si>
-    <t>UI Updates(Add Loading Bar, Bubbled Coversation)</t>
+    <t>Added Bubbled conversation in create / edit conversation + UI styling update</t>
   </si>
   <si>
     <t>Setup Dynamic Inference Pipeline</t>
@@ -1916,7 +1916,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0" outlineLevelRow="2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="26.88"/>
+    <col customWidth="1" min="1" max="1" width="39.38"/>
     <col customWidth="1" min="2" max="2" width="47.63"/>
     <col customWidth="1" min="3" max="3" width="13.38"/>
     <col customWidth="1" min="4" max="4" width="11.0"/>
@@ -2937,21 +2937,21 @@
         <v>35</v>
       </c>
       <c r="D38" s="22">
-        <v>2.0</v>
+        <v>2.5</v>
       </c>
       <c r="E38" s="22">
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
       <c r="F38" s="23" t="s">
         <v>36</v>
       </c>
       <c r="H38" s="20">
         <f t="shared" si="5"/>
-        <v>-0.7</v>
+        <v>-1.3</v>
       </c>
       <c r="I38" s="20">
         <f t="shared" si="6"/>
-        <v>25.92592593</v>
+        <v>34.21052632</v>
       </c>
     </row>
     <row r="39" ht="12.75" customHeight="1">
@@ -2993,21 +2993,21 @@
         <v>80</v>
       </c>
       <c r="D40" s="22">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="E40" s="22">
-        <v>3.5</v>
+        <v>5.2</v>
       </c>
       <c r="F40" s="23" t="s">
         <v>36</v>
       </c>
       <c r="H40" s="20">
         <f t="shared" si="5"/>
-        <v>-0.5</v>
+        <v>-1.2</v>
       </c>
       <c r="I40" s="20">
         <f t="shared" si="6"/>
-        <v>14.28571429</v>
+        <v>23.07692308</v>
       </c>
     </row>
     <row r="41" ht="12.75" customHeight="1">

</xml_diff>